<commit_message>
fix vtb went nahui
</commit_message>
<xml_diff>
--- a/erp_valuation/erp_portfolio.xlsx
+++ b/erp_valuation/erp_portfolio.xlsx
@@ -527,16 +527,16 @@
         <v>19.08913342354207</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>36.52560246505649</v>
+        <v>7.851244304880336</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>12.67486995776239</v>
+        <v>12.23925949930118</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>8.77</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>3.904869957762395</v>
+        <v>3.469259499301183</v>
       </c>
     </row>
     <row r="3">
@@ -555,16 +555,16 @@
         <v>19.68507051261704</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>38.42818955724745</v>
+        <v>8.260208841095547</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>13.23563568622964</v>
+        <v>12.77733465514106</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>8.23</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>5.005635686229642</v>
+        <v>4.547334655141062</v>
       </c>
     </row>
     <row r="4">
@@ -583,16 +583,16 @@
         <v>19.05438378745552</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>38.7031001572502</v>
+        <v>8.319301371730404</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>12.84164802876876</v>
+        <v>12.3800683677762</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>8.43</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>4.411648028768765</v>
+        <v>3.950068367776199</v>
       </c>
     </row>
     <row r="5">
@@ -611,16 +611,16 @@
         <v>18.30785009429028</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>38.86118324239953</v>
+        <v>8.353281616769864</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>12.26905070191468</v>
+        <v>11.80558571554623</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>8.390000000000001</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>3.879050701914684</v>
+        <v>3.415585715546234</v>
       </c>
     </row>
     <row r="6">
@@ -639,16 +639,16 @@
         <v>20.72341951426353</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>35.69351481335104</v>
+        <v>7.672385559350714</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>12.16373494860707</v>
+        <v>11.73804810697836</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>8.25</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>3.913734948607072</v>
+        <v>3.488048106978356</v>
       </c>
     </row>
     <row r="7">
@@ -667,16 +667,16 @@
         <v>21.64834897388687</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>32.85181698154589</v>
+        <v>7.06155747131314</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>11.87581873347102</v>
+        <v>11.48402245659083</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>8.01</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>3.865818733471022</v>
+        <v>3.474022456590832</v>
       </c>
     </row>
     <row r="8">
@@ -695,16 +695,16 @@
         <v>21.26612311808534</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>30.82659908762471</v>
+        <v>6.626233222493365</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>12.01801505636099</v>
+        <v>11.65037186760847</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>7.45</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>4.56801505636099</v>
+        <v>4.200371867608472</v>
       </c>
     </row>
     <row r="9">
@@ -723,16 +723,16 @@
         <v>21.42395840799424</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>31.33766098967614</v>
+        <v>6.736086902573284</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>12.93330963096822</v>
+        <v>12.55957143229307</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>7.43</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>5.503309630968221</v>
+        <v>5.129571432293069</v>
       </c>
     </row>
     <row r="10">
@@ -751,16 +751,16 @@
         <v>20.7929403151282</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>28.45734774223907</v>
+        <v>6.116958361111272</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>12.80664270876458</v>
+        <v>12.46725560875859</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>7.21</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>5.596642708764576</v>
+        <v>5.257255608758594</v>
       </c>
     </row>
     <row r="11">
@@ -782,16 +782,16 @@
         <v>20.4659151974959</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>28.13044156604022</v>
+        <v>6.046689287341252</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>12.57244634425558</v>
+        <v>12.29566940986691</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>7.16</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>5.412446344255576</v>
+        <v>5.135669409866914</v>
       </c>
     </row>
     <row r="12">
@@ -813,16 +813,16 @@
         <v>19.66281621935698</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>28.44248837546238</v>
+        <v>6.113764313350083</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>11.92722156434915</v>
+        <v>11.64737438454345</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>6.51</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>5.417221564349154</v>
+        <v>5.137374384543445</v>
       </c>
     </row>
     <row r="13">
@@ -844,16 +844,16 @@
         <v>19.2824148381953</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>28.08928100347952</v>
+        <v>6.037841749981683</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>11.02849343482321</v>
+        <v>10.75212148143339</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>6.6</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>4.428493434823212</v>
+        <v>4.152121481433392</v>
       </c>
     </row>
     <row r="14">
@@ -875,16 +875,16 @@
         <v>18.02677704153395</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>33.59001883139116</v>
+        <v>7.220235293944389</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>11.25190035142719</v>
+        <v>10.92140634135686</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>6.42</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>4.831900351427194</v>
+        <v>4.50140634135686</v>
       </c>
     </row>
     <row r="15">
@@ -906,16 +906,16 @@
         <v>21.47215262384002</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>35.96992554296213</v>
+        <v>7.731800545557801</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>12.0697548340369</v>
+        <v>11.71584479325076</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>6.37</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>5.699754834036901</v>
+        <v>5.34584479325076</v>
       </c>
     </row>
     <row r="16">
@@ -937,16 +937,16 @@
         <v>27.55484768079231</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>47.80910655756287</v>
+        <v>10.27665391530735</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>15.71711864053564</v>
+        <v>15.24672225810425</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>6.55</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>9.167118640535644</v>
+        <v>8.696722258104248</v>
       </c>
     </row>
     <row r="17">
@@ -968,16 +968,16 @@
         <v>25.80624569777168</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>44.65836314545987</v>
+        <v>9.599395920888814</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>14.65598331052775</v>
+        <v>14.21658726275516</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>6.89</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>7.765983310527754</v>
+        <v>7.326587262755161</v>
       </c>
     </row>
     <row r="18">
@@ -999,16 +999,16 @@
         <v>17.80772152671224</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>41.50045448142646</v>
+        <v>8.920597742609777</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>12.69115153117262</v>
+        <v>12.28282631735969</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>6.18</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>6.51115153117262</v>
+        <v>6.102826317359694</v>
       </c>
     </row>
     <row r="19">
@@ -1030,16 +1030,16 @@
         <v>18.51648656260129</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>42.99233957833366</v>
+        <v>9.241281142201457</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>12.11145768561761</v>
+        <v>11.68845373373323</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>5.67</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>6.441457685617607</v>
+        <v>6.018453733733232</v>
       </c>
     </row>
     <row r="20">
@@ -1061,16 +1061,16 @@
         <v>18.77070562720411</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>38.88224750923997</v>
+        <v>8.357809419021057</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>10.7292973145386</v>
+        <v>10.34673278058047</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>6.01</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>4.719297314538604</v>
+        <v>4.336732780580475</v>
       </c>
     </row>
     <row r="21">
@@ -1092,16 +1092,16 @@
         <v>10.71995641599881</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>36.44658651758898</v>
+        <v>7.834259684075175</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>9.50443568650768</v>
+        <v>9.145835752639334</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>6.01</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>3.49443568650768</v>
+        <v>3.135835752639334</v>
       </c>
     </row>
     <row r="22">
@@ -1123,16 +1123,16 @@
         <v>10.44565988107247</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>37.39805650644554</v>
+        <v>8.038779878873365</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>9.288357051010799</v>
+        <v>8.920395552516448</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>6.22</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>3.068357051010799</v>
+        <v>2.700395552516448</v>
       </c>
     </row>
     <row r="23">
@@ -1154,16 +1154,16 @@
         <v>11.43707185377575</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>39.47031985488167</v>
+        <v>8.484216633220857</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>10.45137515672191</v>
+        <v>10.06302454718287</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>6.39</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>4.061375156721913</v>
+        <v>3.673024547182872</v>
       </c>
     </row>
     <row r="24">
@@ -1188,16 +1188,16 @@
         <v>5.667647954234813</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>27.59912057863434</v>
+        <v>5.932480880226692</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>8.773424047949756</v>
+        <v>8.517832735490186</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>6.52</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>2.253424047949757</v>
+        <v>1.997832735490187</v>
       </c>
     </row>
     <row r="25">
@@ -1222,16 +1222,16 @@
         <v>5.855223524312912</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>27.10023160657036</v>
+        <v>5.825243793461807</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>8.242749223068996</v>
+        <v>7.991778046485789</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>6.16</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>2.082749223068996</v>
+        <v>1.831778046485788</v>
       </c>
     </row>
     <row r="26">
@@ -1256,16 +1256,16 @@
         <v>3.411173174992418</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>15.79581090058082</v>
+        <v>3.395338119139771</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>8.044208804510866</v>
+        <v>7.897926171050143</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>6.25</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>1.794208804510866</v>
+        <v>1.647926171050143</v>
       </c>
     </row>
     <row r="27">
@@ -1290,16 +1290,16 @@
         <v>3.082994003575836</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>15.6083488157189</v>
+        <v>3.355042804981403</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>7.543511555381165</v>
+        <v>7.398964980146275</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>6.58</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>0.9635115553811646</v>
+        <v>0.8189649801462746</v>
       </c>
     </row>
     <row r="28">
@@ -1324,16 +1324,16 @@
         <v>2.817822060376203</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>13.54745481312837</v>
+        <v>2.912049912084408</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>6.940927847197894</v>
+        <v>6.815466901936662</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>7.02</v>
       </c>
       <c r="K28" s="4" t="n">
-        <v>-0.07907215280210522</v>
+        <v>-0.2045330980633375</v>
       </c>
     </row>
     <row r="29">
@@ -1358,16 +1358,16 @@
         <v>3.072134256990506</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>11.21471961904609</v>
+        <v>2.410624263462897</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>6.810067482216238</v>
+        <v>6.706209647393882</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>7.27</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>-0.4599325177837619</v>
+        <v>-0.5637903526061177</v>
       </c>
     </row>
     <row r="30">
@@ -1392,16 +1392,16 @@
         <v>5.61092328242254</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>19.04004040775008</v>
+        <v>4.092691118758473</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>7.823409438198516</v>
+        <v>7.647082482300239</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>7.17</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0.6534094381985165</v>
+        <v>0.4770824823002391</v>
       </c>
     </row>
     <row r="31">
@@ -1426,16 +1426,16 @@
         <v>5.219966092926011</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>19.14805507741756</v>
+        <v>4.115909067343487</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>7.80871180876252</v>
+        <v>7.631384545223767</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>7.26</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0.54871180876252</v>
+        <v>0.3713845452237674</v>
       </c>
     </row>
     <row r="32">
@@ -1460,16 +1460,16 @@
         <v>5.475931372413843</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>19.15398204452778</v>
+        <v>4.117183079642499</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>7.856170133185644</v>
+        <v>7.678787980894248</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>7.21</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>0.6461701331856435</v>
+        <v>0.4687879808942483</v>
       </c>
     </row>
     <row r="33">
@@ -1494,16 +1494,16 @@
         <v>11.26399397667822</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>29.82906832118022</v>
+        <v>6.411812180253669</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>8.54687111950769</v>
+        <v>8.270628595767322</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>6.97</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>1.576871119507691</v>
+        <v>1.300628595767322</v>
       </c>
     </row>
     <row r="34">
@@ -1528,16 +1528,16 @@
         <v>9.783457615293401</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>30.4179138734853</v>
+        <v>6.538385596624072</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>8.215557513275504</v>
+        <v>7.93386177927357</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>7.09</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>1.125557513275504</v>
+        <v>0.8438617792735696</v>
       </c>
     </row>
     <row r="35">
@@ -1562,16 +1562,16 @@
         <v>9.448934422190694</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>29.80644054320095</v>
+        <v>6.406948298455638</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>7.795708855541113</v>
+        <v>7.519675884255697</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>7.45</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>0.3457088555411127</v>
+        <v>0.06967588425569726</v>
       </c>
     </row>
     <row r="36">
@@ -1596,16 +1596,16 @@
         <v>14.38422404715066</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>44.71345187576364</v>
+        <v>9.61123734309326</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>9.31695817628888</v>
+        <v>8.902873610914304</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>8.32</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.9969581762888797</v>
+        <v>0.5828736109143033</v>
       </c>
     </row>
     <row r="37">
@@ -1630,16 +1630,16 @@
         <v>13.59417234239063</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>43.78569065829785</v>
+        <v>9.411813391581832</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>9.915587737926296</v>
+        <v>9.510095029909841</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>8.35</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>1.565587737926297</v>
+        <v>1.160095029909842</v>
       </c>
     </row>
     <row r="38">
@@ -1664,16 +1664,16 @@
         <v>17.28644177708432</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>57.33042542138138</v>
+        <v>12.32327862399001</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>11.14856196313792</v>
+        <v>10.61763349983536</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>8.369999999999999</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>2.778561963137925</v>
+        <v>2.247633499835365</v>
       </c>
     </row>
     <row r="39">
@@ -1698,16 +1698,16 @@
         <v>32.38646722938399</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>124.8098470884176</v>
+        <v>26.82810234501654</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>23.16944856119304</v>
+        <v>22.01360330393863</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>9.42</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>13.74944856119304</v>
+        <v>12.59360330393863</v>
       </c>
     </row>
     <row r="40">
@@ -1732,10 +1732,10 @@
         <v>22.79637161894582</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>126.7639406539433</v>
+        <v>27.24813829082235</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>21.53419143678171</v>
+        <v>20.36024961236827</v>
       </c>
     </row>
     <row r="41">
@@ -1760,16 +1760,16 @@
         <v>24.3848718417819</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>124.9030119406856</v>
+        <v>26.84812829849628</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>23.80685488204624</v>
+        <v>22.65014683908102</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>11.36</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>12.44685488204624</v>
+        <v>11.29014683908102</v>
       </c>
     </row>
     <row r="42">
@@ -1794,16 +1794,16 @@
         <v>27.38071406266658</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>137.0795207508507</v>
+        <v>29.46549088794553</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>24.69749487544833</v>
+        <v>23.42802201234696</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>10.32</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>14.37749487544833</v>
+        <v>13.10802201234696</v>
       </c>
     </row>
     <row r="43">
@@ -1828,16 +1828,16 @@
         <v>28.49559475949014</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>141.1656931916804</v>
+        <v>30.34382104377292</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>23.66815123381252</v>
+        <v>22.36083694115864</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>9.23</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>14.43815123381252</v>
+        <v>13.13083694115864</v>
       </c>
     </row>
     <row r="44">
@@ -1862,16 +1862,16 @@
         <v>29.24229235587904</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>135.0511716410049</v>
+        <v>29.02949357860009</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>23.24448639124682</v>
+        <v>21.99379776475309</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>8.84</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>14.40448639124682</v>
+        <v>13.15379776475309</v>
       </c>
     </row>
     <row r="45">
@@ -1896,16 +1896,16 @@
         <v>26.79398253243592</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>129.7454652338112</v>
+        <v>27.88902239122681</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>22.52579701007567</v>
+        <v>21.32424373411878</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>8.869999999999999</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>13.65579701007568</v>
+        <v>12.45424373411878</v>
       </c>
     </row>
     <row r="46">
@@ -1930,16 +1930,16 @@
         <v>37.34211540214511</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>168.1129286636354</v>
+        <v>36.13617804141209</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>27.28260609787113</v>
+        <v>25.72573750286871</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>9.08</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>18.20260609787113</v>
+        <v>16.64573750286871</v>
       </c>
     </row>
     <row r="47">
@@ -1964,16 +1964,16 @@
         <v>29.53035511211866</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>149.0454884173442</v>
+        <v>32.03759727780775</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>23.92132737649255</v>
+        <v>22.54103948317983</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>10.5</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>13.42132737649255</v>
+        <v>12.04103948317983</v>
       </c>
     </row>
     <row r="48">
@@ -1998,16 +1998,16 @@
         <v>24.41325895330124</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>148.1656449201934</v>
+        <v>31.84847332693522</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>22.02667943851863</v>
+        <v>20.65453964374968</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>10.23</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>11.79667943851863</v>
+        <v>10.42453964374968</v>
       </c>
     </row>
     <row r="49">
@@ -2032,16 +2032,16 @@
         <v>22.46567685563094</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>153.1376464275825</v>
+        <v>32.91721404260419</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>21.54544778378352</v>
+        <v>20.12726302945856</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>10.24</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>11.30544778378352</v>
+        <v>9.887263029458561</v>
       </c>
     </row>
     <row r="50">
@@ -2066,16 +2066,16 @@
         <v>22.51248721679747</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>148.0782315603585</v>
+        <v>31.82968366715531</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>19.37530274124448</v>
+        <v>18.00397246847833</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>10.27</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>9.105302741244476</v>
+        <v>7.733972468478335</v>
       </c>
     </row>
     <row r="51">
@@ -2100,16 +2100,16 @@
         <v>21.4038225980015</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>152.4863927671979</v>
+        <v>32.77722589053965</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>18.25786051509935</v>
+        <v>16.84570692315609</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>10.65</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>7.607860515099349</v>
+        <v>6.195706923156086</v>
       </c>
     </row>
     <row r="52">
@@ -2134,16 +2134,16 @@
         <v>20.13948547945324</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>82.6249415966674</v>
+        <v>29.7416283438965</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>14.05834290542251</v>
+        <v>13.43450295471342</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>10.82</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>3.23834290542251</v>
+        <v>2.614502954713416</v>
       </c>
     </row>
     <row r="53">
@@ -2168,16 +2168,16 @@
         <v>19.47976134871442</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>67.45348517387698</v>
+        <v>24.28051926904962</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>12.47808167422522</v>
+        <v>11.96879019331329</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>10.82</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>1.658081674225219</v>
+        <v>1.148790193313294</v>
       </c>
     </row>
     <row r="54">
@@ -2202,16 +2202,16 @@
         <v>19.28624202847321</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>80.40277291845889</v>
+        <v>28.94173773377847</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>14.15220303988944</v>
+        <v>13.54514104474548</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>10.91</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>3.242203039889441</v>
+        <v>2.635141044745483</v>
       </c>
     </row>
     <row r="55">
@@ -2236,16 +2236,16 @@
         <v>17.9967607277201</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>66.53587918087359</v>
+        <v>29.62907898039576</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>14.30093107386747</v>
+        <v>13.8655586472601</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>10.89</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>3.410931073867468</v>
+        <v>2.975558647260101</v>
       </c>
     </row>
     <row r="56">
@@ -2270,16 +2270,16 @@
         <v>17.06287476563301</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>55.89116947655409</v>
+        <v>24.88888544218021</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>12.87130955692517</v>
+        <v>12.505589972537</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>11.08</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>1.791309556925173</v>
+        <v>1.425589972536995</v>
       </c>
     </row>
     <row r="57">
@@ -2304,16 +2304,16 @@
         <v>17.5257728321209</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>57.43255792919773</v>
+        <v>25.57528082411689</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>13.86709144841647</v>
+        <v>13.49128590680891</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>11.21</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>2.657091448416468</v>
+        <v>2.281285906808913</v>
       </c>
     </row>
     <row r="58">
@@ -2338,16 +2338,16 @@
         <v>18.15076082045445</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>64.41608880580253</v>
+        <v>28.68511555467585</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>14.3733238675815</v>
+        <v>13.95182212684851</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>11.47</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>2.903323867581502</v>
+        <v>2.481822126848513</v>
       </c>
     </row>
     <row r="59">
@@ -2372,16 +2372,16 @@
         <v>16.96450885142118</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>65.39575280699682</v>
+        <v>29.1213695340774</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>13.89504808043625</v>
+        <v>13.46713598338557</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>11.97</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>1.925048080436246</v>
+        <v>1.497135983385574</v>
       </c>
     </row>
     <row r="60">
@@ -2406,16 +2406,16 @@
         <v>20.8800453075799</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>69.23304521315475</v>
+        <v>30.83015344394131</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>14.8543829237674</v>
+        <v>14.40136179791846</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>12.23</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>2.624382923767405</v>
+        <v>2.171361797918458</v>
       </c>
     </row>
     <row r="61">
@@ -2440,16 +2440,16 @@
         <v>20.56677422997123</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>72.91143231552915</v>
+        <v>32.46817526492672</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>15.23088888351344</v>
+        <v>14.75379851354422</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>11.88</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>3.350888883513443</v>
+        <v>2.873798513544216</v>
       </c>
     </row>
     <row r="62">
@@ -2474,16 +2474,16 @@
         <v>20.79110483818339</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>65.50085153380275</v>
+        <v>29.1681710269803</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>16.11074430416497</v>
+        <v>15.68214450164943</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>11.74</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>4.370744304164974</v>
+        <v>3.942144501649427</v>
       </c>
     </row>
     <row r="63">
@@ -2508,16 +2508,16 @@
         <v>20.68319252933468</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>68.71647498156682</v>
+        <v>30.60011965797399</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>15.45588528673661</v>
+        <v>15.00624429861198</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>11.71</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>3.745885286736611</v>
+        <v>3.296244298611976</v>
       </c>
     </row>
     <row r="64">
@@ -2542,16 +2542,16 @@
         <v>21.13103894291727</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>70.21519853623566</v>
+        <v>31.26751594277168</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>15.01210023936496</v>
+        <v>14.55265246851133</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>12.3</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>2.712100239364963</v>
+        <v>2.252652468511329</v>
       </c>
     </row>
     <row r="65">
@@ -2576,16 +2576,16 @@
         <v>20.54104000335987</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>68.89293500719891</v>
+        <v>30.67869903650935</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>14.70308827917611</v>
+        <v>14.25229263839632</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>13.36</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>1.343088279176106</v>
+        <v>0.8922926383963254</v>
       </c>
     </row>
     <row r="66">
@@ -2610,16 +2610,16 @@
         <v>22.76473490916588</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>75.97652302826364</v>
+        <v>33.83309019395038</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>15.47115490670867</v>
+        <v>14.97400835054631</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>13.61</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1.861154906708666</v>
+        <v>1.364008350546312</v>
       </c>
     </row>
     <row r="67">
@@ -2644,16 +2644,16 @@
         <v>22.41838069382961</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>71.03481445854452</v>
+        <v>31.63249894434386</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>14.79969349884931</v>
+        <v>14.33488263401729</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>14.96</v>
       </c>
       <c r="K67" s="4" t="n">
-        <v>-0.1603065011506946</v>
+        <v>-0.6251173659827156</v>
       </c>
     </row>
     <row r="68">
@@ -2678,16 +2678,16 @@
         <v>24.56049944216917</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>76.75710374430747</v>
+        <v>31.88374803839209</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>16.30641030179403</v>
+        <v>15.77706011002511</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>15.14</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>1.166410301794027</v>
+        <v>0.6370601100251108</v>
       </c>
     </row>
     <row r="69">
@@ -2712,16 +2712,16 @@
         <v>27.5225196590493</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>84.5398532226926</v>
+        <v>35.116585278335</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>18.6367054465879</v>
+        <v>18.05368204767719</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>15.42</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>3.216705446587904</v>
+        <v>2.633682047677192</v>
       </c>
     </row>
     <row r="70">
@@ -2746,16 +2746,16 @@
         <v>25.81117654662714</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>86.86628970922069</v>
+        <v>36.08295205281462</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>17.64818925425947</v>
+        <v>17.04912174294473</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>15.88</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>1.768189254259473</v>
+        <v>1.169121742944727</v>
       </c>
     </row>
     <row r="71">
@@ -2780,16 +2780,16 @@
         <v>30.16952540833589</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>102.7734986420189</v>
+        <v>42.6905677244131</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>19.85829963524305</v>
+        <v>19.14952912982974</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>15.87</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>3.988299635243051</v>
+        <v>3.279529129829738</v>
       </c>
     </row>
     <row r="72">
@@ -2814,16 +2814,16 @@
         <v>22.14796142562243</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>114.3308816633844</v>
+        <v>47.49133104482092</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>20.1311061344782</v>
+        <v>19.34263091614233</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>16.84</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>3.291106134478198</v>
+        <v>2.50263091614233</v>
       </c>
     </row>
     <row r="73">
@@ -2848,16 +2848,16 @@
         <v>17.46840287343869</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>99.28772054985896</v>
+        <v>41.24262785974076</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>17.05434103174768</v>
+        <v>16.36960995997031</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>16.17</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>0.8843410317476774</v>
+        <v>0.1996099599703065</v>
       </c>
     </row>
     <row r="74">
@@ -2882,16 +2882,16 @@
         <v>19.41566696816943</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>118.826351702471</v>
+        <v>49.35868177913012</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>17.65080348545137</v>
+        <v>16.831325561031</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>15.38</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>2.270803485451369</v>
+        <v>1.451325561031004</v>
       </c>
     </row>
     <row r="75">
@@ -2916,16 +2916,16 @@
         <v>18.3943410823337</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>108.7060266556194</v>
+        <v>45.15485075737434</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>16.11049445719776</v>
+        <v>15.36081067225093</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>16.6</v>
       </c>
       <c r="K75" s="4" t="n">
-        <v>-0.4895055428022417</v>
+        <v>-1.239189327749072</v>
       </c>
     </row>
     <row r="76">
@@ -2950,16 +2950,16 @@
         <v>20.85254507407065</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>121.6244832152306</v>
+        <v>50.52098358286025</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>16.19689586503241</v>
+        <v>15.35812081525662</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>15.55</v>
       </c>
-      <c r="K76" s="3" t="n">
-        <v>0.6468958650324126</v>
+      <c r="K76" s="4" t="n">
+        <v>-0.1918791847433852</v>
       </c>
     </row>
     <row r="77">
@@ -2984,16 +2984,16 @@
         <v>22.5042318126109</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>101.6140942336422</v>
+        <v>42.20896854690343</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>16.32928020965052</v>
+        <v>15.62850545858401</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>15.22</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>1.109280209650519</v>
+        <v>0.4085054585840133</v>
       </c>
     </row>
     <row r="78">
@@ -3018,16 +3018,16 @@
         <v>18.88663129780421</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>109.847831303558</v>
+        <v>45.62913925873848</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>16.6534233454286</v>
+        <v>15.89586518169642</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>15.79</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>0.863423345428604</v>
+        <v>0.1058651816964247</v>
       </c>
     </row>
     <row r="79">
@@ -3052,16 +3052,16 @@
         <v>18.23971186718758</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>97.10705478633119</v>
+        <v>40.33681205418513</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>16.21855499968541</v>
+        <v>15.54886274234733</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>15.41</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>0.8085549996854127</v>
+        <v>0.1388627423473263</v>
       </c>
     </row>
     <row r="80">
@@ -3086,16 +3086,16 @@
         <v>19.22417385644482</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>132.6309805761103</v>
+        <v>55.09291727395582</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>17.16161574815813</v>
+        <v>16.24693513128206</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>14.7</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>2.461615748158128</v>
+        <v>1.546935131282062</v>
       </c>
     </row>
     <row r="81">
@@ -3120,16 +3120,16 @@
         <v>11.41095129815538</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>133.4141152827802</v>
+        <v>55.41821966877728</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>17.41698395445769</v>
+        <v>16.49690250186826</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>14.1</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>3.316983954457688</v>
+        <v>2.396902501868263</v>
       </c>
     </row>
     <row r="82">
@@ -3154,16 +3154,16 @@
         <v>12.7520293128997</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>119.3211636384267</v>
+        <v>61.10151420347143</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>18.49856537603772</v>
+        <v>17.8117751391968</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>13.85</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>4.648565376037718</v>
+        <v>3.961775139196797</v>
       </c>
     </row>
     <row r="83">
@@ -3185,16 +3185,16 @@
         <v>13.71730908439518</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>119.5667526256273</v>
+        <v>61.22727445028835</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19.82360512411116</v>
+        <v>19.09243309684751</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>14.95</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>4.873605124111158</v>
+        <v>4.142433096847512</v>
       </c>
     </row>
     <row r="84">
@@ -3219,16 +3219,16 @@
         <v>10.13451644820684</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>111.1210180252848</v>
+        <v>56.90241575040731</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>18.2958187361679</v>
+        <v>17.65622699937551</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>14.58</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>3.715818736167895</v>
+        <v>3.076226999375509</v>
       </c>
     </row>
     <row r="85">
@@ -3253,16 +3253,16 @@
         <v>10.03540137291876</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>112.0903650393519</v>
+        <v>57.39879517332002</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>18.17584496613211</v>
+        <v>17.53067384974711</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>14.35</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>3.825844966132115</v>
+        <v>3.180673849747107</v>
       </c>
     </row>
     <row r="86">
@@ -3287,16 +3287,16 @@
         <v>6.780199126557799</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>94.31581935820005</v>
+        <v>48.29687542764808</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>18.7531948993332</v>
+        <v>18.21033073391868</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>14.35</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>4.403194899333199</v>
+        <v>3.860330733918678</v>
       </c>
     </row>
     <row r="87">
@@ -3321,16 +3321,16 @@
         <v>7.012368278640311</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>84.05690567362392</v>
+        <v>43.04353108288635</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>18.09768133655067</v>
+        <v>17.61386555404088</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>14.63</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>3.467681336550667</v>
+        <v>2.983865554040884</v>
       </c>
     </row>
     <row r="88">
@@ -3355,16 +3355,16 @@
         <v>5.73871550358888</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>84.91657302202056</v>
+        <v>43.48374617211803</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>18.64996207344997</v>
+        <v>18.16119820693056</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>14.31</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>4.339962073449973</v>
+        <v>3.85119820693056</v>
       </c>
     </row>
     <row r="89">

</xml_diff>